<commit_message>
Fixtures anonimizados: identificadores reales de IDM sustituidos por inventados
Los fixtures de la Fase 1 usaban ejemplos reales del contexto (albarán, pedido, registro, códigos de artículo y de
proveedor en Siddex, referencias de proveedor). Se sustituyen por valores inventados con la misma forma en fixtures,
golden, tests y documentación, y se regeneran los PDF, exports de Siddex e imágenes sintéticas. El mapa de productos
versionado pasa a ser un ejemplo; el real vive en datos/mapa_productos.csv y calcular_mes/generar_pedidos lo usan si
existe. Nuevo test guardián con huellas SHA-256 que falla si un identificador real vuelve a un fichero versionado.
El historial conserva los valores antiguos: reescribirlo queda a decisión de Oliver.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/ficticios/siddex/articulos.xlsx
+++ b/fixtures/ficticios/siddex/articulos.xlsx
@@ -706,7 +706,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>134.000.842</t>
+          <t>900.000.842</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -740,7 +740,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>I33.000.786</t>
+          <t>Z33.000.786</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -836,12 +836,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MO01001</t>
+          <t>SV09001</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SERVICIO TURISMO (CONTRATOS)</t>
+          <t>SERVICIO FICTICIO (CONTRATOS)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">

</xml_diff>